<commit_message>
waxan badalay gant charka qaybta dateka oo wax ka khaldanayeen
</commit_message>
<xml_diff>
--- a/gentchart_srms.xlsx
+++ b/gentchart_srms.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xamppp\htdocs\srms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F231B85-720C-4124-973D-67286ACD00E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98CB3713-31CB-46A6-8D50-4F60880D0D76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{76D0844D-04C0-4B41-B09F-3DB426E6ADAF}"/>
   </bookViews>
@@ -1131,7 +1131,7 @@
         <v>4</v>
       </c>
       <c r="D10" s="6">
-        <v>46202</v>
+        <v>46201</v>
       </c>
       <c r="E10" s="6">
         <v>46205</v>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="K10" s="3" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>x</v>
       </c>
       <c r="L10" s="3" t="str">
         <f t="shared" si="0"/>

</xml_diff>

<commit_message>
last change in the system
</commit_message>
<xml_diff>
--- a/gentchart_srms.xlsx
+++ b/gentchart_srms.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xamppp\htdocs\srms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98CB3713-31CB-46A6-8D50-4F60880D0D76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEE26B04-AC2E-494F-A4FF-EB7EFF78AE5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{76D0844D-04C0-4B41-B09F-3DB426E6ADAF}"/>
   </bookViews>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
   <si>
     <t>Project Name</t>
   </si>
@@ -104,6 +104,15 @@
   </si>
   <si>
     <t>System Integration</t>
+  </si>
+  <si>
+    <t>Testing</t>
+  </si>
+  <si>
+    <t>Bug Fixing</t>
+  </si>
+  <si>
+    <t>Final Deployment</t>
   </si>
 </sst>
 </file>
@@ -206,7 +215,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -257,11 +266,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="16" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -284,11 +306,35 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="16" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color theme="9" tint="-0.499984740745262"/>
@@ -609,7 +655,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9821937D-D706-4AA5-9617-AFC912A992FA}">
-  <dimension ref="A2:AQ21"/>
+  <dimension ref="A2:BI22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.44140625" customWidth="1"/>
@@ -619,7 +665,7 @@
     <col min="5" max="5" width="14.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:61" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -633,24 +679,23 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:43" ht="18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="B3" s="11" t="s">
         <v>4</v>
       </c>
       <c r="C3" s="11">
         <f>E3-D3</f>
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="D3" s="12">
         <f>MIN(D8:D15)</f>
         <v>46196</v>
       </c>
       <c r="E3" s="12">
-        <f>MAX(E8:E15)</f>
-        <v>46233</v>
+        <v>46249</v>
       </c>
     </row>
-    <row r="7" spans="1:43" ht="34.200000000000003" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:61" ht="36.6" x14ac:dyDescent="0.35">
       <c r="A7" s="13" t="s">
         <v>5</v>
       </c>
@@ -780,8 +825,62 @@
       <c r="AQ7" s="2">
         <v>46233</v>
       </c>
+      <c r="AR7" s="2">
+        <v>46234</v>
+      </c>
+      <c r="AS7" s="2">
+        <v>46235</v>
+      </c>
+      <c r="AT7" s="2">
+        <v>46236</v>
+      </c>
+      <c r="AU7" s="2">
+        <v>46237</v>
+      </c>
+      <c r="AV7" s="2">
+        <v>46238</v>
+      </c>
+      <c r="AW7" s="2">
+        <v>46239</v>
+      </c>
+      <c r="AX7" s="2">
+        <v>46240</v>
+      </c>
+      <c r="AY7" s="2">
+        <v>46241</v>
+      </c>
+      <c r="AZ7" s="2">
+        <v>46242</v>
+      </c>
+      <c r="BA7" s="2">
+        <v>46243</v>
+      </c>
+      <c r="BB7" s="2">
+        <v>46244</v>
+      </c>
+      <c r="BC7" s="2">
+        <v>46245</v>
+      </c>
+      <c r="BD7" s="2">
+        <v>46246</v>
+      </c>
+      <c r="BE7" s="2">
+        <v>46247</v>
+      </c>
+      <c r="BF7" s="2">
+        <v>46248</v>
+      </c>
+      <c r="BG7" s="2">
+        <v>46249</v>
+      </c>
+      <c r="BH7" s="2">
+        <v>46250</v>
+      </c>
+      <c r="BI7" s="2">
+        <v>46251</v>
+      </c>
     </row>
-    <row r="8" spans="1:43" ht="18" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A8" s="4" cm="1">
         <f t="array" ref="A8:A17">_xlfn.SEQUENCE(10,)</f>
         <v>1</v>
@@ -950,8 +1049,80 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
+      <c r="AR8" s="3" t="str">
+        <f t="shared" ref="AR8:BI18" si="1">IF(AND(AR$7&gt;=$D8,AR$7&lt;=$E8),"x","")</f>
+        <v/>
+      </c>
+      <c r="AS8" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AT8" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AU8" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AV8" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AW8" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AX8" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AY8" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AZ8" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="BA8" s="3" t="str">
+        <f t="shared" ref="BA8:BI22" si="2">IF(AND(BA$7&gt;=$D8,BA$7&lt;=$E8),"x","")</f>
+        <v/>
+      </c>
+      <c r="BB8" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BC8" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BD8" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BE8" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BF8" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BG8" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BH8" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BI8" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
-    <row r="9" spans="1:43" ht="18" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A9" s="4">
         <v>2</v>
       </c>
@@ -959,76 +1130,78 @@
         <v>9</v>
       </c>
       <c r="C9" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D9" s="6">
+        <f>E8+1</f>
         <v>46199</v>
       </c>
       <c r="E9" s="6">
-        <v>46200</v>
+        <f>D9+C9</f>
+        <v>46201</v>
       </c>
       <c r="F9" s="3" t="str">
-        <f t="shared" ref="F9:U15" si="1">IF(AND(F$7&gt;=$D9,F$7&lt;=$E9),"x","")</f>
+        <f t="shared" ref="F9:U18" si="3">IF(AND(F$7&gt;=$D9,F$7&lt;=$E9),"x","")</f>
         <v/>
       </c>
       <c r="G9" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="H9" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="I9" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>x</v>
       </c>
       <c r="J9" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>x</v>
       </c>
       <c r="K9" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v/>
+        <f t="shared" si="3"/>
+        <v>x</v>
       </c>
       <c r="L9" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="M9" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="N9" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="O9" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="P9" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="Q9" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="R9" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="S9" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="T9" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="U9" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="V9" s="3" t="str">
@@ -1119,8 +1292,80 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
+      <c r="AR9" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AS9" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AT9" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AU9" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AV9" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AW9" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AX9" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AY9" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AZ9" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="BA9" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BB9" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BC9" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BD9" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BE9" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BF9" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BG9" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BH9" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BI9" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
-    <row r="10" spans="1:43" ht="18" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A10" s="4">
         <v>3</v>
       </c>
@@ -1131,13 +1376,14 @@
         <v>4</v>
       </c>
       <c r="D10" s="6">
-        <v>46201</v>
+        <f>E9+1</f>
+        <v>46202</v>
       </c>
       <c r="E10" s="6">
         <v>46205</v>
       </c>
       <c r="F10" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G10" s="3" t="str">
@@ -1158,7 +1404,7 @@
       </c>
       <c r="K10" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>x</v>
+        <v/>
       </c>
       <c r="L10" s="3" t="str">
         <f t="shared" si="0"/>
@@ -1288,8 +1534,80 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
+      <c r="AR10" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AS10" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AT10" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AU10" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AV10" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AW10" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AX10" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AY10" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AZ10" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="BA10" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BB10" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BC10" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BD10" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BE10" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BF10" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BG10" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BH10" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BI10" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
-    <row r="11" spans="1:43" ht="18" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A11" s="4">
         <v>4</v>
       </c>
@@ -1300,15 +1618,15 @@
         <v>5</v>
       </c>
       <c r="D11" s="6">
-        <f>E10</f>
-        <v>46205</v>
+        <f>E10+1</f>
+        <v>46206</v>
       </c>
       <c r="E11" s="6">
         <f>D11+C11</f>
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="F11" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G11" s="3" t="str">
@@ -1345,7 +1663,7 @@
       </c>
       <c r="O11" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>x</v>
+        <v/>
       </c>
       <c r="P11" s="3" t="str">
         <f t="shared" si="0"/>
@@ -1369,7 +1687,7 @@
       </c>
       <c r="U11" s="3" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>x</v>
       </c>
       <c r="V11" s="3" t="str">
         <f t="shared" si="0"/>
@@ -1459,8 +1777,80 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
+      <c r="AR11" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AS11" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AT11" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AU11" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AV11" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AW11" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AX11" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AY11" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AZ11" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="BA11" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BB11" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BC11" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BD11" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BE11" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BF11" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BG11" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BH11" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BI11" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
-    <row r="12" spans="1:43" ht="18" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A12" s="4">
         <v>5</v>
       </c>
@@ -1471,15 +1861,15 @@
         <v>5</v>
       </c>
       <c r="D12" s="6">
-        <f t="shared" ref="D12:D15" si="2">E11</f>
-        <v>46210</v>
+        <f t="shared" ref="D12:D18" si="4">E11+1</f>
+        <v>46212</v>
       </c>
       <c r="E12" s="6">
-        <f t="shared" ref="E12:E15" si="3">D12+C12</f>
-        <v>46215</v>
+        <f t="shared" ref="E12:E18" si="5">D12+C12</f>
+        <v>46217</v>
       </c>
       <c r="F12" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G12" s="3" t="str">
@@ -1536,11 +1926,11 @@
       </c>
       <c r="T12" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>x</v>
+        <v/>
       </c>
       <c r="U12" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>x</v>
+        <v/>
       </c>
       <c r="V12" s="3" t="str">
         <f t="shared" si="0"/>
@@ -1560,11 +1950,11 @@
       </c>
       <c r="Z12" s="3" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>x</v>
       </c>
       <c r="AA12" s="3" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>x</v>
       </c>
       <c r="AB12" s="3" t="str">
         <f t="shared" si="0"/>
@@ -1630,8 +2020,80 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
+      <c r="AR12" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AS12" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AT12" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AU12" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AV12" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AW12" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AX12" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AY12" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AZ12" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="BA12" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BB12" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BC12" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BD12" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BE12" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BF12" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BG12" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BH12" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BI12" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
-    <row r="13" spans="1:43" ht="18" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A13" s="4">
         <v>6</v>
       </c>
@@ -1642,15 +2104,15 @@
         <v>6</v>
       </c>
       <c r="D13" s="6">
-        <f t="shared" si="2"/>
-        <v>46215</v>
+        <f t="shared" si="4"/>
+        <v>46218</v>
       </c>
       <c r="E13" s="6">
-        <f t="shared" si="3"/>
-        <v>46221</v>
+        <f t="shared" si="5"/>
+        <v>46224</v>
       </c>
       <c r="F13" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G13" s="3" t="str">
@@ -1727,15 +2189,15 @@
       </c>
       <c r="Y13" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>x</v>
+        <v/>
       </c>
       <c r="Z13" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>x</v>
+        <v/>
       </c>
       <c r="AA13" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>x</v>
+        <v/>
       </c>
       <c r="AB13" s="3" t="str">
         <f t="shared" si="0"/>
@@ -1755,15 +2217,15 @@
       </c>
       <c r="AF13" s="3" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>x</v>
       </c>
       <c r="AG13" s="3" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>x</v>
       </c>
       <c r="AH13" s="3" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>x</v>
       </c>
       <c r="AI13" s="3" t="str">
         <f t="shared" si="0"/>
@@ -1801,8 +2263,80 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
+      <c r="AR13" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AS13" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AT13" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AU13" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AV13" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AW13" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AX13" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AY13" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AZ13" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="BA13" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BB13" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BC13" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BD13" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BE13" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BF13" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BG13" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BH13" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BI13" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
-    <row r="14" spans="1:43" ht="18" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A14" s="4">
         <v>7</v>
       </c>
@@ -1813,15 +2347,15 @@
         <v>6</v>
       </c>
       <c r="D14" s="6">
-        <f t="shared" si="2"/>
-        <v>46221</v>
+        <f t="shared" si="4"/>
+        <v>46225</v>
       </c>
       <c r="E14" s="6">
-        <f t="shared" si="3"/>
-        <v>46227</v>
+        <f t="shared" si="5"/>
+        <v>46231</v>
       </c>
       <c r="F14" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G14" s="3" t="str">
@@ -1922,19 +2456,19 @@
       </c>
       <c r="AE14" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>x</v>
+        <v/>
       </c>
       <c r="AF14" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>x</v>
+        <v/>
       </c>
       <c r="AG14" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>x</v>
+        <v/>
       </c>
       <c r="AH14" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>x</v>
+        <v/>
       </c>
       <c r="AI14" s="3" t="str">
         <f t="shared" si="0"/>
@@ -1950,19 +2484,19 @@
       </c>
       <c r="AL14" s="3" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>x</v>
       </c>
       <c r="AM14" s="3" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>x</v>
       </c>
       <c r="AN14" s="3" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>x</v>
       </c>
       <c r="AO14" s="3" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>x</v>
       </c>
       <c r="AP14" s="3" t="str">
         <f t="shared" si="0"/>
@@ -1972,8 +2506,80 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
+      <c r="AR14" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AS14" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AT14" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AU14" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AV14" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AW14" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AX14" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AY14" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AZ14" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="BA14" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BB14" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BC14" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BD14" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BE14" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BF14" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BG14" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BH14" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BI14" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
-    <row r="15" spans="1:43" ht="18" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A15" s="4">
         <v>8</v>
       </c>
@@ -1984,15 +2590,15 @@
         <v>6</v>
       </c>
       <c r="D15" s="6">
-        <f t="shared" si="2"/>
-        <v>46227</v>
+        <f t="shared" si="4"/>
+        <v>46232</v>
       </c>
       <c r="E15" s="6">
-        <f t="shared" si="3"/>
-        <v>46233</v>
+        <f t="shared" si="5"/>
+        <v>46238</v>
       </c>
       <c r="F15" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G15" s="3" t="str">
@@ -2040,170 +2646,1291 @@
         <v/>
       </c>
       <c r="R15" s="3" t="str">
-        <f t="shared" ref="R15:AQ15" si="4">IF(AND(R$7&gt;=$D15,R$7&lt;=$E15),"x","")</f>
+        <f t="shared" ref="R15:AR18" si="6">IF(AND(R$7&gt;=$D15,R$7&lt;=$E15),"x","")</f>
         <v/>
       </c>
       <c r="S15" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="T15" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="U15" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="V15" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="W15" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="X15" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="Y15" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="Z15" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AA15" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AB15" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AC15" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AD15" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AE15" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AF15" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AG15" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AH15" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AI15" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AJ15" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="AK15" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>x</v>
+        <f t="shared" si="6"/>
+        <v/>
       </c>
       <c r="AL15" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>x</v>
+        <f t="shared" si="6"/>
+        <v/>
       </c>
       <c r="AM15" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>x</v>
+        <f t="shared" si="6"/>
+        <v/>
       </c>
       <c r="AN15" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>x</v>
+        <f t="shared" si="6"/>
+        <v/>
       </c>
       <c r="AO15" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>x</v>
+        <f t="shared" si="6"/>
+        <v/>
       </c>
       <c r="AP15" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>x</v>
       </c>
       <c r="AQ15" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>x</v>
+        <f t="shared" si="6"/>
+        <v>x</v>
+      </c>
+      <c r="AR15" s="3" t="str">
+        <f t="shared" si="6"/>
+        <v>x</v>
+      </c>
+      <c r="AS15" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>x</v>
+      </c>
+      <c r="AT15" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>x</v>
+      </c>
+      <c r="AU15" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>x</v>
+      </c>
+      <c r="AV15" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>x</v>
+      </c>
+      <c r="AW15" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AX15" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AY15" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AZ15" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="BA15" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BB15" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BC15" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BD15" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BE15" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BF15" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BG15" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BH15" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BI15" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v/>
       </c>
     </row>
-    <row r="16" spans="1:43" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A16" s="4">
         <v>9</v>
       </c>
-      <c r="B16" s="8"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
+      <c r="B16" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16" s="4">
+        <v>3</v>
+      </c>
+      <c r="D16" s="6">
+        <f t="shared" si="4"/>
+        <v>46239</v>
+      </c>
+      <c r="E16" s="6">
+        <f t="shared" si="5"/>
+        <v>46242</v>
+      </c>
+      <c r="F16" s="15" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="G16" s="15" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="H16" s="15" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I16" s="15" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="J16" s="15" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="K16" s="15" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="L16" s="15" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="M16" s="15" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="N16" s="15" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="O16" s="15" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="P16" s="15" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="Q16" s="15" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="R16" s="15" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="S16" s="15" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="T16" s="15" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="U16" s="15" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="V16" s="15" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="W16" s="15" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="X16" s="15" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="Y16" s="15" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="Z16" s="15" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AA16" s="15" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AB16" s="15" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AC16" s="15" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AD16" s="15" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AE16" s="15" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AF16" s="15" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AG16" s="15" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AH16" s="15" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AI16" s="15" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AJ16" s="15" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AK16" s="15" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AL16" s="15" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AM16" s="15" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AN16" s="15" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AO16" s="15" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AP16" s="15" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AQ16" s="15" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AR16" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AS16" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AT16" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AU16" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AV16" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AW16" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v>x</v>
+      </c>
+      <c r="AX16" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v>x</v>
+      </c>
+      <c r="AY16" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v>x</v>
+      </c>
+      <c r="AZ16" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v>x</v>
+      </c>
+      <c r="BA16" s="15" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BB16" s="15" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BC16" s="15" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BD16" s="15" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BE16" s="15" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BF16" s="15" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BG16" s="15" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BH16" s="15" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BI16" s="15" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
-    <row r="17" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A17" s="4">
         <v>10</v>
       </c>
-      <c r="B17" s="8"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
+      <c r="B17" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C17" s="4">
+        <v>2</v>
+      </c>
+      <c r="D17" s="6">
+        <f t="shared" si="4"/>
+        <v>46243</v>
+      </c>
+      <c r="E17" s="6">
+        <f t="shared" si="5"/>
+        <v>46245</v>
+      </c>
+      <c r="F17" s="16" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="G17" s="16" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="H17" s="16" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I17" s="16" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="J17" s="16" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="K17" s="16" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="L17" s="16" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="M17" s="16" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="N17" s="16" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="O17" s="16" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="P17" s="16" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="Q17" s="16" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="R17" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="S17" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="T17" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="U17" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="V17" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="W17" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="X17" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="Y17" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="Z17" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AA17" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AB17" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AC17" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AD17" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AE17" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AF17" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AG17" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AH17" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AI17" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AJ17" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AK17" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AL17" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AM17" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AN17" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AO17" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AP17" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AQ17" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AR17" s="16" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AS17" s="16" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AT17" s="16" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AU17" s="16" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AV17" s="16" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AW17" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AX17" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AY17" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AZ17" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="BA17" s="16" t="str">
+        <f>IF(AND(BA$7&gt;=$D17,BA$7&lt;=$E17),"x","")</f>
+        <v>x</v>
+      </c>
+      <c r="BB17" s="16" t="str">
+        <f t="shared" si="2"/>
+        <v>x</v>
+      </c>
+      <c r="BC17" s="16" t="str">
+        <f t="shared" si="2"/>
+        <v>x</v>
+      </c>
+      <c r="BD17" s="16" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BE17" s="16" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BF17" s="16" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BG17" s="16" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BH17" s="16" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="BI17" s="16" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
-    <row r="18" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:61" ht="18" x14ac:dyDescent="0.35">
       <c r="A18" s="4">
         <v>11</v>
       </c>
-      <c r="B18" s="9"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
+      <c r="B18" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="C18" s="4">
+        <v>3</v>
+      </c>
+      <c r="D18" s="6">
+        <f t="shared" si="4"/>
+        <v>46246</v>
+      </c>
+      <c r="E18" s="6">
+        <f t="shared" si="5"/>
+        <v>46249</v>
+      </c>
+      <c r="F18" s="16" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="G18" s="16" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="H18" s="16" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I18" s="16" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="J18" s="16" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="K18" s="16" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="L18" s="16" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="M18" s="16" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="N18" s="16" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="O18" s="16" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="P18" s="16" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="Q18" s="16" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="R18" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="S18" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="T18" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="U18" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="V18" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="W18" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="X18" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="Y18" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="Z18" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AA18" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AB18" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AC18" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AD18" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AE18" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AF18" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AG18" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AH18" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AI18" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AJ18" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AK18" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AL18" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AM18" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AN18" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AO18" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AP18" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AQ18" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="AR18" s="16" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AS18" s="16" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AT18" s="16" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AU18" s="16" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AV18" s="16" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AW18" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AX18" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AY18" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="AZ18" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="BA18" s="16" t="str">
+        <f t="shared" ref="BA18:BI22" si="7">IF(AND(BA$7&gt;=$D18,BA$7&lt;=$E18),"x","")</f>
+        <v/>
+      </c>
+      <c r="BB18" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BC18" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BD18" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v>x</v>
+      </c>
+      <c r="BE18" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v>x</v>
+      </c>
+      <c r="BF18" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v>x</v>
+      </c>
+      <c r="BG18" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v>x</v>
+      </c>
+      <c r="BH18" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BI18" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
     </row>
-    <row r="19" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:61" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A19" s="10">
         <v>12</v>
       </c>
       <c r="B19" s="8"/>
       <c r="C19" s="9"/>
       <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="16"/>
+      <c r="G19" s="16"/>
+      <c r="H19" s="16"/>
+      <c r="I19" s="16"/>
+      <c r="J19" s="16"/>
+      <c r="K19" s="16"/>
+      <c r="L19" s="16"/>
+      <c r="M19" s="16"/>
+      <c r="N19" s="16"/>
+      <c r="O19" s="16"/>
+      <c r="P19" s="16"/>
+      <c r="Q19" s="16"/>
+      <c r="R19" s="16"/>
+      <c r="S19" s="16"/>
+      <c r="T19" s="16"/>
+      <c r="U19" s="16"/>
+      <c r="V19" s="16"/>
+      <c r="W19" s="16"/>
+      <c r="X19" s="16"/>
+      <c r="Y19" s="16"/>
+      <c r="Z19" s="16"/>
+      <c r="AA19" s="16"/>
+      <c r="AB19" s="16"/>
+      <c r="AC19" s="16"/>
+      <c r="AD19" s="16"/>
+      <c r="AE19" s="16"/>
+      <c r="AF19" s="16"/>
+      <c r="AG19" s="16"/>
+      <c r="AH19" s="16"/>
+      <c r="AI19" s="16"/>
+      <c r="AJ19" s="16"/>
+      <c r="AK19" s="16"/>
+      <c r="AL19" s="16"/>
+      <c r="AM19" s="16"/>
+      <c r="AN19" s="16"/>
+      <c r="AO19" s="16"/>
+      <c r="AP19" s="16"/>
+      <c r="AQ19" s="16"/>
+      <c r="AR19" s="16"/>
+      <c r="AS19" s="16"/>
+      <c r="AT19" s="16"/>
+      <c r="AU19" s="16"/>
+      <c r="AV19" s="16"/>
+      <c r="AW19" s="16"/>
+      <c r="AX19" s="16"/>
+      <c r="AY19" s="16"/>
+      <c r="AZ19" s="16"/>
+      <c r="BA19" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BB19" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BC19" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BD19" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BE19" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BF19" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BG19" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BH19" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BI19" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
     </row>
-    <row r="20" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:61" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" s="10">
         <v>13</v>
       </c>
       <c r="B20" s="8"/>
       <c r="C20" s="9"/>
       <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="16"/>
+      <c r="I20" s="16"/>
+      <c r="J20" s="16"/>
+      <c r="K20" s="16"/>
+      <c r="L20" s="16"/>
+      <c r="M20" s="16"/>
+      <c r="N20" s="16"/>
+      <c r="O20" s="16"/>
+      <c r="P20" s="16"/>
+      <c r="Q20" s="16"/>
+      <c r="R20" s="16"/>
+      <c r="S20" s="16"/>
+      <c r="T20" s="16"/>
+      <c r="U20" s="16"/>
+      <c r="V20" s="16"/>
+      <c r="W20" s="16"/>
+      <c r="X20" s="16"/>
+      <c r="Y20" s="16"/>
+      <c r="Z20" s="16"/>
+      <c r="AA20" s="16"/>
+      <c r="AB20" s="16"/>
+      <c r="AC20" s="16"/>
+      <c r="AD20" s="16"/>
+      <c r="AE20" s="16"/>
+      <c r="AF20" s="16"/>
+      <c r="AG20" s="16"/>
+      <c r="AH20" s="16"/>
+      <c r="AI20" s="16"/>
+      <c r="AJ20" s="16"/>
+      <c r="AK20" s="16"/>
+      <c r="AL20" s="16"/>
+      <c r="AM20" s="16"/>
+      <c r="AN20" s="16"/>
+      <c r="AO20" s="16"/>
+      <c r="AP20" s="16"/>
+      <c r="AQ20" s="16"/>
+      <c r="AR20" s="16"/>
+      <c r="AS20" s="16"/>
+      <c r="AT20" s="16"/>
+      <c r="AU20" s="16"/>
+      <c r="AV20" s="16"/>
+      <c r="AW20" s="16"/>
+      <c r="AX20" s="16"/>
+      <c r="AY20" s="16"/>
+      <c r="AZ20" s="16"/>
+      <c r="BA20" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BB20" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BC20" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BD20" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BE20" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BF20" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BG20" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BH20" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BI20" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
     </row>
-    <row r="21" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:61" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" s="10">
         <v>14</v>
       </c>
       <c r="B21" s="8"/>
       <c r="C21" s="9"/>
       <c r="D21" s="9"/>
-      <c r="E21" s="9"/>
+      <c r="E21" s="14"/>
+      <c r="F21" s="16"/>
+      <c r="G21" s="16"/>
+      <c r="H21" s="16"/>
+      <c r="I21" s="16"/>
+      <c r="J21" s="16"/>
+      <c r="K21" s="16"/>
+      <c r="L21" s="16"/>
+      <c r="M21" s="16"/>
+      <c r="N21" s="16"/>
+      <c r="O21" s="16"/>
+      <c r="P21" s="16"/>
+      <c r="Q21" s="16"/>
+      <c r="R21" s="16"/>
+      <c r="S21" s="16"/>
+      <c r="T21" s="16"/>
+      <c r="U21" s="16"/>
+      <c r="V21" s="16"/>
+      <c r="W21" s="16"/>
+      <c r="X21" s="16"/>
+      <c r="Y21" s="16"/>
+      <c r="Z21" s="16"/>
+      <c r="AA21" s="16"/>
+      <c r="AB21" s="16"/>
+      <c r="AC21" s="16"/>
+      <c r="AD21" s="16"/>
+      <c r="AE21" s="16"/>
+      <c r="AF21" s="16"/>
+      <c r="AG21" s="16"/>
+      <c r="AH21" s="16"/>
+      <c r="AI21" s="16"/>
+      <c r="AJ21" s="16"/>
+      <c r="AK21" s="16"/>
+      <c r="AL21" s="16"/>
+      <c r="AM21" s="16"/>
+      <c r="AN21" s="16"/>
+      <c r="AO21" s="16"/>
+      <c r="AP21" s="16"/>
+      <c r="AQ21" s="16"/>
+      <c r="AR21" s="16"/>
+      <c r="AS21" s="16"/>
+      <c r="AT21" s="16"/>
+      <c r="AU21" s="16"/>
+      <c r="AV21" s="16"/>
+      <c r="AW21" s="16"/>
+      <c r="AX21" s="16"/>
+      <c r="AY21" s="16"/>
+      <c r="AZ21" s="16"/>
+      <c r="BA21" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BB21" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BC21" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BD21" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BE21" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BF21" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BG21" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BH21" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BI21" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="22" spans="1:61" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A22" s="10">
+        <v>15</v>
+      </c>
+      <c r="B22" s="8"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="14"/>
+      <c r="F22" s="16"/>
+      <c r="G22" s="16"/>
+      <c r="H22" s="16"/>
+      <c r="I22" s="16"/>
+      <c r="J22" s="16"/>
+      <c r="K22" s="16"/>
+      <c r="L22" s="16"/>
+      <c r="M22" s="16"/>
+      <c r="N22" s="16"/>
+      <c r="O22" s="16"/>
+      <c r="P22" s="16"/>
+      <c r="Q22" s="16"/>
+      <c r="R22" s="16"/>
+      <c r="S22" s="16"/>
+      <c r="T22" s="16"/>
+      <c r="U22" s="16"/>
+      <c r="V22" s="16"/>
+      <c r="W22" s="16"/>
+      <c r="X22" s="16"/>
+      <c r="Y22" s="16"/>
+      <c r="Z22" s="16"/>
+      <c r="AA22" s="16"/>
+      <c r="AB22" s="16"/>
+      <c r="AC22" s="16"/>
+      <c r="AD22" s="16"/>
+      <c r="AE22" s="16"/>
+      <c r="AF22" s="16"/>
+      <c r="AG22" s="16"/>
+      <c r="AH22" s="16"/>
+      <c r="AI22" s="16"/>
+      <c r="AJ22" s="16"/>
+      <c r="AK22" s="16"/>
+      <c r="AL22" s="16"/>
+      <c r="AM22" s="16"/>
+      <c r="AN22" s="16"/>
+      <c r="AO22" s="16"/>
+      <c r="AP22" s="16"/>
+      <c r="AQ22" s="16"/>
+      <c r="AR22" s="16"/>
+      <c r="AS22" s="16"/>
+      <c r="AT22" s="16"/>
+      <c r="AU22" s="16"/>
+      <c r="AV22" s="16"/>
+      <c r="AW22" s="16"/>
+      <c r="AX22" s="16"/>
+      <c r="AY22" s="16"/>
+      <c r="AZ22" s="16"/>
+      <c r="BA22" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BB22" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BC22" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BD22" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BE22" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BF22" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BG22" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BH22" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="BI22" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F8:AQ15">
+  <conditionalFormatting sqref="AW17:AZ18 F8:BI16">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="BA17:BI22">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>